<commit_message>
Add Team Install Performance (Weekly) card
</commit_message>
<xml_diff>
--- a/Dashboard_Template_30_Slides_Final_WK31.xlsx
+++ b/Dashboard_Template_30_Slides_Final_WK31.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_Dashboad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{604AF303-7065-4090-B27E-953EE239C9A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66D67757-06ED-4720-BC80-060D53A128C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="863" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="863" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part 1 - Overview" sheetId="1" r:id="rId1"/>
@@ -5580,21 +5580,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -5617,6 +5602,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6754,7 +6754,7 @@
         <v>1362</v>
       </c>
       <c r="D11" s="66">
-        <v>169361.5</v>
+        <v>53878.640000000043</v>
       </c>
       <c r="E11" s="65" t="s">
         <v>1363</v>
@@ -7358,7 +7358,7 @@
       </c>
       <c r="D44" s="77">
         <f>SUM(D8:D13)</f>
-        <v>1092793.1399999999</v>
+        <v>977310.27999999991</v>
       </c>
       <c r="E44" t="s">
         <v>1359</v>
@@ -7469,17 +7469,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="88" t="s">
         <v>1315</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="82"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="90"/>
       <c r="D1" s="50"/>
-      <c r="E1" s="80" t="s">
+      <c r="E1" s="88" t="s">
         <v>1316</v>
       </c>
-      <c r="F1" s="81"/>
-      <c r="G1" s="82"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="90"/>
     </row>
     <row r="2" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="51" t="s">
@@ -7589,24 +7589,24 @@
     <row r="7" spans="1:7" ht="16.5" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="78" t="s">
+      <c r="A22" s="86" t="s">
         <v>134</v>
       </c>
-      <c r="B22" s="79"/>
+      <c r="B22" s="87"/>
       <c r="C22" s="57"/>
       <c r="D22" s="58"/>
-      <c r="E22" s="78" t="s">
+      <c r="E22" s="86" t="s">
         <v>135</v>
       </c>
-      <c r="F22" s="79"/>
+      <c r="F22" s="87"/>
       <c r="G22" s="59" t="s">
         <v>1327</v>
       </c>
       <c r="H22" s="58"/>
-      <c r="I22" s="78" t="s">
+      <c r="I22" s="86" t="s">
         <v>136</v>
       </c>
-      <c r="J22" s="79"/>
+      <c r="J22" s="87"/>
       <c r="K22" s="76" t="s">
         <v>1327</v>
       </c>
@@ -7641,18 +7641,18 @@
       </c>
     </row>
     <row r="24" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="83" t="s">
+      <c r="A24" s="78" t="s">
         <v>988</v>
       </c>
-      <c r="B24" s="84" t="s">
+      <c r="B24" s="79" t="s">
         <v>1534</v>
       </c>
       <c r="C24" s="57"/>
       <c r="D24" s="62"/>
-      <c r="E24" s="83" t="s">
+      <c r="E24" s="78" t="s">
         <v>972</v>
       </c>
-      <c r="F24" s="84" t="s">
+      <c r="F24" s="79" t="s">
         <v>1341</v>
       </c>
       <c r="G24" s="72" t="s">
@@ -7662,24 +7662,24 @@
       <c r="I24" s="68" t="s">
         <v>892</v>
       </c>
-      <c r="J24" s="87" t="s">
+      <c r="J24" s="82" t="s">
         <v>1341</v>
       </c>
-      <c r="K24" s="88" t="s">
+      <c r="K24" s="83" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="85" t="s">
+      <c r="A25" s="80" t="s">
         <v>1241</v>
       </c>
-      <c r="B25" s="86" t="s">
+      <c r="B25" s="81" t="s">
         <v>1374</v>
       </c>
-      <c r="E25" s="83" t="s">
+      <c r="E25" s="78" t="s">
         <v>996</v>
       </c>
-      <c r="F25" s="84" t="s">
+      <c r="F25" s="79" t="s">
         <v>1341</v>
       </c>
       <c r="G25" s="72" t="s">
@@ -7688,24 +7688,24 @@
       <c r="I25" s="70" t="s">
         <v>1117</v>
       </c>
-      <c r="J25" s="89" t="s">
+      <c r="J25" s="84" t="s">
         <v>1340</v>
       </c>
-      <c r="K25" s="90" t="s">
+      <c r="K25" s="85" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="85" t="s">
+      <c r="A26" s="80" t="s">
         <v>1249</v>
       </c>
-      <c r="B26" s="86" t="s">
+      <c r="B26" s="81" t="s">
         <v>1535</v>
       </c>
-      <c r="E26" s="83" t="s">
+      <c r="E26" s="78" t="s">
         <v>992</v>
       </c>
-      <c r="F26" s="84" t="s">
+      <c r="F26" s="79" t="s">
         <v>1341</v>
       </c>
       <c r="G26" s="72" t="s">
@@ -7716,16 +7716,16 @@
       <c r="K26" s="72"/>
     </row>
     <row r="27" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A27" s="85" t="s">
+      <c r="A27" s="80" t="s">
         <v>1173</v>
       </c>
-      <c r="B27" s="86" t="s">
+      <c r="B27" s="81" t="s">
         <v>1536</v>
       </c>
-      <c r="E27" s="83" t="s">
+      <c r="E27" s="78" t="s">
         <v>984</v>
       </c>
-      <c r="F27" s="84" t="s">
+      <c r="F27" s="79" t="s">
         <v>1329</v>
       </c>
       <c r="G27" s="72" t="s">
@@ -7736,16 +7736,16 @@
       <c r="K27" s="72"/>
     </row>
     <row r="28" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="85" t="s">
+      <c r="A28" s="80" t="s">
         <v>1181</v>
       </c>
-      <c r="B28" s="86" t="s">
+      <c r="B28" s="81" t="s">
         <v>1537</v>
       </c>
-      <c r="E28" s="83" t="s">
+      <c r="E28" s="78" t="s">
         <v>1221</v>
       </c>
-      <c r="F28" s="84" t="s">
+      <c r="F28" s="79" t="s">
         <v>1341</v>
       </c>
       <c r="G28" s="72" t="s">
@@ -7756,16 +7756,16 @@
       <c r="K28" s="72"/>
     </row>
     <row r="29" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A29" s="85" t="s">
+      <c r="A29" s="80" t="s">
         <v>1189</v>
       </c>
-      <c r="B29" s="86" t="s">
+      <c r="B29" s="81" t="s">
         <v>1374</v>
       </c>
-      <c r="E29" s="83" t="s">
+      <c r="E29" s="78" t="s">
         <v>1233</v>
       </c>
-      <c r="F29" s="84" t="s">
+      <c r="F29" s="79" t="s">
         <v>1375</v>
       </c>
       <c r="G29" s="72" t="s">
@@ -7776,16 +7776,16 @@
       <c r="K29" s="72"/>
     </row>
     <row r="30" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A30" s="85" t="s">
+      <c r="A30" s="80" t="s">
         <v>1201</v>
       </c>
-      <c r="B30" s="86" t="s">
+      <c r="B30" s="81" t="s">
         <v>1535</v>
       </c>
-      <c r="E30" s="83" t="s">
+      <c r="E30" s="78" t="s">
         <v>1209</v>
       </c>
-      <c r="F30" s="84" t="s">
+      <c r="F30" s="79" t="s">
         <v>1340</v>
       </c>
       <c r="G30" s="72" t="s">
@@ -7796,16 +7796,16 @@
       <c r="K30" s="72"/>
     </row>
     <row r="31" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A31" s="85" t="s">
+      <c r="A31" s="80" t="s">
         <v>1205</v>
       </c>
-      <c r="B31" s="86" t="s">
+      <c r="B31" s="81" t="s">
         <v>1374</v>
       </c>
-      <c r="E31" s="83" t="s">
+      <c r="E31" s="78" t="s">
         <v>1133</v>
       </c>
-      <c r="F31" s="84" t="s">
+      <c r="F31" s="79" t="s">
         <v>1534</v>
       </c>
       <c r="G31" s="72" t="s">
@@ -7816,16 +7816,16 @@
       <c r="K31" s="72"/>
     </row>
     <row r="32" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="85" t="s">
+      <c r="A32" s="80" t="s">
         <v>1229</v>
       </c>
-      <c r="B32" s="86" t="s">
+      <c r="B32" s="81" t="s">
         <v>1537</v>
       </c>
-      <c r="E32" s="83" t="s">
+      <c r="E32" s="78" t="s">
         <v>1121</v>
       </c>
-      <c r="F32" s="84" t="s">
+      <c r="F32" s="79" t="s">
         <v>1329</v>
       </c>
       <c r="G32" s="72" t="s">
@@ -7836,16 +7836,16 @@
       <c r="K32" s="72"/>
     </row>
     <row r="33" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A33" s="85" t="s">
+      <c r="A33" s="80" t="s">
         <v>1113</v>
       </c>
-      <c r="B33" s="86" t="s">
+      <c r="B33" s="81" t="s">
         <v>1535</v>
       </c>
-      <c r="E33" s="83" t="s">
+      <c r="E33" s="78" t="s">
         <v>1125</v>
       </c>
-      <c r="F33" s="84" t="s">
+      <c r="F33" s="79" t="s">
         <v>1534</v>
       </c>
       <c r="G33" s="72" t="s">
@@ -7856,16 +7856,16 @@
       <c r="K33" s="72"/>
     </row>
     <row r="34" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="83" t="s">
+      <c r="A34" s="78" t="s">
         <v>1383</v>
       </c>
-      <c r="B34" s="84" t="s">
+      <c r="B34" s="79" t="s">
         <v>1329</v>
       </c>
-      <c r="E34" s="83" t="s">
+      <c r="E34" s="78" t="s">
         <v>1392</v>
       </c>
-      <c r="F34" s="84" t="s">
+      <c r="F34" s="79" t="s">
         <v>1538</v>
       </c>
       <c r="G34" s="72" t="s">
@@ -7876,16 +7876,16 @@
       <c r="K34" s="72"/>
     </row>
     <row r="35" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="85" t="s">
+      <c r="A35" s="80" t="s">
         <v>1389</v>
       </c>
-      <c r="B35" s="86" t="s">
+      <c r="B35" s="81" t="s">
         <v>1341</v>
       </c>
-      <c r="E35" s="83" t="s">
+      <c r="E35" s="78" t="s">
         <v>1395</v>
       </c>
-      <c r="F35" s="84" t="s">
+      <c r="F35" s="79" t="s">
         <v>1329</v>
       </c>
       <c r="G35" s="72" t="s">
@@ -7896,16 +7896,16 @@
       <c r="K35" s="73"/>
     </row>
     <row r="36" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A36" s="83" t="s">
+      <c r="A36" s="78" t="s">
         <v>1422</v>
       </c>
-      <c r="B36" s="84" t="s">
+      <c r="B36" s="79" t="s">
         <v>1329</v>
       </c>
-      <c r="E36" s="83" t="s">
+      <c r="E36" s="78" t="s">
         <v>1410</v>
       </c>
-      <c r="F36" s="84" t="s">
+      <c r="F36" s="79" t="s">
         <v>1340</v>
       </c>
       <c r="G36" s="72" t="s">
@@ -7913,16 +7913,16 @@
       </c>
     </row>
     <row r="37" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A37" s="83" t="s">
+      <c r="A37" s="78" t="s">
         <v>1425</v>
       </c>
-      <c r="B37" s="84" t="s">
+      <c r="B37" s="79" t="s">
         <v>1534</v>
       </c>
-      <c r="E37" s="83" t="s">
+      <c r="E37" s="78" t="s">
         <v>1413</v>
       </c>
-      <c r="F37" s="84" t="s">
+      <c r="F37" s="79" t="s">
         <v>1329</v>
       </c>
       <c r="G37" s="72" t="s">
@@ -7930,10 +7930,10 @@
       </c>
     </row>
     <row r="38" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="85" t="s">
+      <c r="A38" s="80" t="s">
         <v>1428</v>
       </c>
-      <c r="B38" s="86" t="s">
+      <c r="B38" s="81" t="s">
         <v>1341</v>
       </c>
       <c r="E38" s="67" t="s">
@@ -7947,10 +7947,10 @@
       </c>
     </row>
     <row r="39" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A39" s="85" t="s">
+      <c r="A39" s="80" t="s">
         <v>1431</v>
       </c>
-      <c r="B39" s="86" t="s">
+      <c r="B39" s="81" t="s">
         <v>1341</v>
       </c>
     </row>

</xml_diff>